<commit_message>
CRV Q28: FIX swapped CRV/PCL click labels in Action.Both (control arm disambiguates: crv_click=0 for control)
CRV and PCL click columns were reversed. Correct: Android Both CRV 21430/PCL 45199,
iOS Both CRV 67177/PCL 130326. PCL is the more-clicked banner ~2:1, not CRV.
Removes false 'PCL clicks halve' click-stage cannibalization signal (was swap artifact).

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/campaigns/CRV/bulletproof_analysis/journey_table.xlsx
+++ b/campaigns/CRV/bulletproof_analysis/journey_table.xlsx
@@ -616,16 +616,16 @@
         <v>0.5840212836410555</v>
       </c>
       <c r="E4" s="7" t="n">
+        <v>21430</v>
+      </c>
+      <c r="F4" s="8" t="n">
+        <v>0.2094901071400641</v>
+      </c>
+      <c r="G4" s="7" t="n">
         <v>45199</v>
       </c>
-      <c r="F4" s="8" t="n">
+      <c r="H4" s="9" t="n">
         <v>0.4418452334402127</v>
-      </c>
-      <c r="G4" s="7" t="n">
-        <v>21430</v>
-      </c>
-      <c r="H4" s="9" t="n">
-        <v>0.2094901071400641</v>
       </c>
     </row>
     <row r="5">
@@ -701,16 +701,16 @@
         <v>0.835083717264403</v>
       </c>
       <c r="E9" s="7" t="n">
+        <v>67177</v>
+      </c>
+      <c r="F9" s="8" t="n">
+        <v>0.1718204884237234</v>
+      </c>
+      <c r="G9" s="7" t="n">
         <v>130326</v>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="H9" s="9" t="n">
         <v>0.3333384487891716</v>
-      </c>
-      <c r="G9" s="7" t="n">
-        <v>67177</v>
-      </c>
-      <c r="H9" s="9" t="n">
-        <v>0.1718204884237234</v>
       </c>
     </row>
     <row r="10">

</xml_diff>